<commit_message>
Pre-publication cleanup: fix bugs, correct docs, redact node/GPU identifiers
</commit_message>
<xml_diff>
--- a/analysis/aesrc_validation/review_sheet.xlsx
+++ b/analysis/aesrc_validation/review_sheet.xlsx
@@ -171,15 +171,21 @@
     <comment ref="AF1" authorId="0" shapeId="0">
       <text>
         <t>Free text. Pick from these, comma-separated if more than one applies:
-- Noise / audio quality
-- Speed (fast or slow / unclear)
+- Reference error
+- Misalignment
+- Truncated audio
+- Disfluency
+- Number formatting
+- Technical vocabulary
+- Acronym or code
+- Hindi named entity
+- Indian-language named entity
+- Foreign named entity
+- English name or rare word
+- Brand or product name
 - Accent / pronunciation
-- Technical vocabulary (jargon, numbers, names)
-- Disfluency (fillers, repetitions, false starts)
-- Code-switching (non-English words)
-- Reference error
-- Misalignment (wrong clip boundary)
-- Other</t>
+- Spelling variant
+- Short utterance</t>
       </text>
     </comment>
     <comment ref="AG1" authorId="0" shapeId="0">

</xml_diff>